<commit_message>
implementar provincia y pais y modal para empresas
</commit_message>
<xml_diff>
--- a/projecto_centralizar/frontend/public/templates/empresas_import_template.xlsx
+++ b/projecto_centralizar/frontend/public/templates/empresas_import_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t xml:space="preserve">empresa</t>
   </si>
@@ -55,6 +55,12 @@
     <t xml:space="preserve">producto</t>
   </si>
   <si>
+    <t xml:space="preserve">provincia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pais</t>
+  </si>
+  <si>
     <t xml:space="preserve">facebook</t>
   </si>
   <si>
@@ -88,6 +94,12 @@
     <t xml:space="preserve">servidores</t>
   </si>
   <si>
+    <t xml:space="preserve">pontevedra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">españa</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.facebook.com/acme</t>
   </si>
   <si>
@@ -119,6 +131,9 @@
   </si>
   <si>
     <t xml:space="preserve">alta tecnologia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lugo</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.facebook.com/techcorp</t>
@@ -354,10 +369,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6.81"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.39"/>
@@ -365,10 +380,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="30.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="13.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="20.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="19.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="32.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="20.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="21.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="21.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -405,10 +422,10 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="0" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -416,23 +433,29 @@
       </c>
       <c r="O1" s="1" t="s">
         <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>6201</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>500</v>
@@ -444,42 +467,48 @@
         <v>500000</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="M2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="L2" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="M2" s="0" t="s">
         <v>25</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C3" s="1" t="n">
         <v>6201</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>100</v>
@@ -491,35 +520,41 @@
         <v>100000</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>24</v>
+        <v>36</v>
+      </c>
+      <c r="L3" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="acme@acme.com"/>
     <hyperlink ref="E2" r:id="rId2" display="www.acme.com"/>
-    <hyperlink ref="L2" r:id="rId3" display="https://www.facebook.com/acme"/>
+    <hyperlink ref="N2" r:id="rId3" display="https://www.facebook.com/acme"/>
     <hyperlink ref="D3" r:id="rId4" display="techcorp@techcorp.com"/>
     <hyperlink ref="E3" r:id="rId5" display="www.techcorp.com"/>
-    <hyperlink ref="L3" r:id="rId6" display="https://www.facebook.com/techcorp"/>
+    <hyperlink ref="N3" r:id="rId6" display="https://www.facebook.com/techcorp"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>